<commit_message>
feat: Add autonomous scan evaluation results, logs, and research paper drafts, updating existing evaluation scripts.
</commit_message>
<xml_diff>
--- a/research/results/Evaluation Form.xlsx
+++ b/research/results/Evaluation Form.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -520,11 +520,11 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -543,11 +543,11 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -566,11 +566,11 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -589,23 +589,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" t="inlineStr">
         <is>
-          <t>Insecure Deserialization</t>
+          <t>Mass Assignment</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -616,53 +616,53 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mass Assignment</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Race Condition</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -674,23 +674,23 @@
     <row r="9">
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sensitive Data Exposure</t>
+          <t>Insecure Deserialization</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
@@ -701,14 +701,14 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -718,51 +718,43 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Social Media (5003)</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SQL Injection</t>
+          <t>SAML Bypass</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cross-Site Scripting (XSS)</t>
+          <t>Information Disclosure</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -772,78 +764,86 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Social Media (5003)</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Insecure Direct Object Reference (IDOR)</t>
+          <t>SQL Injection</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cross-Site Request Forgery (CSRF)</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="C15" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Insecure Direct Object Reference (IDOR)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
         <is>
-          <t>Path Traversal</t>
+          <t>Cross-Site Request Forgery (CSRF)</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -854,19 +854,19 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="C17" t="inlineStr">
         <is>
-          <t>Weak Password</t>
+          <t>Path Traversal</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -877,7 +877,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -889,41 +889,41 @@
     <row r="18">
       <c r="C18" t="inlineStr">
         <is>
-          <t>Session Fixation</t>
+          <t>File Upload</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="C19" t="inlineStr">
         <is>
-          <t>Weak Reset Token</t>
+          <t>Weak Password</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -935,7 +935,7 @@
     <row r="20">
       <c r="C20" t="inlineStr">
         <is>
-          <t>OAuth Bypass</t>
+          <t>Session Fixation</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>
-          <t>JWT Bypass</t>
+          <t>Weak Reset Token</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -969,7 +969,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -979,151 +979,151 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OAuth Bypass</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>3</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Banking (5004)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Insecure Direct Object Reference (IDOR)</t>
-        </is>
-      </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="C24" t="inlineStr">
         <is>
+          <t>Insecure Direct Object Reference (IDOR)</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Cross-Site Request Forgery (CSRF)</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="n">
+    <row r="26">
+      <c r="A26" t="n">
         <v>4</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Blog (5005)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Cross-Site Scripting (XSS)</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>4</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
       <c r="C26" t="inlineStr">
         <is>
-          <t>Server-Side Request Forgery (SSRF)</t>
+          <t>SQL Injection</t>
         </is>
       </c>
       <c r="D26" t="n">
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="C27" t="inlineStr">
         <is>
-          <t>JWT Bypass</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1133,28 +1133,20 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>5</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>File Share (5006)</t>
-        </is>
-      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Cross-Site Scripting (XSS)</t>
+          <t>Broken Access Control (BAC)</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1166,53 +1158,61 @@
     <row r="29">
       <c r="C29" t="inlineStr">
         <is>
-          <t>Insecure Direct Object Reference (IDOR)</t>
+          <t>Server-Side Request Forgery (SSRF)</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="C30" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>JWT Bypass</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="31">
+      <c r="A31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>File Share (5006)</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Path Traversal</t>
+          <t>Cross-Site Scripting (XSS)</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1235,21 +1235,90 @@
     <row r="32">
       <c r="C32" t="inlineStr">
         <is>
+          <t>Insecure Direct Object Reference (IDOR)</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Path Traversal</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>File Upload</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" t="inlineStr">
+        <is>
           <t>Command Injection</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>

</xml_diff>